<commit_message>
Update game doc + xlsx: murphy cutscene, partner float, weight tuning
xlsx: events 17→19, event rules updated, murphy weight system
and profit fly animation added to special mechanics sheet.

md: murphy threshold/probability cap, fullscreen cutscene,
partner hover float panel, deferred event escalation, xlsx sync.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VentureTown_企劃書.xlsx
+++ b/VentureTown_企劃書.xlsx
@@ -3935,7 +3935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3948,14 +3948,14 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>市場事件一覽（每 3 回合觸發，共 17 種）</t>
+          <t>市場事件一覽（每 3 回合觸發，共 19 種）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>事件規則：每 3 回合（第 3、6、9 回合）觸發一次。提前預告，觸發前 1 回合以藍色高亮受影響格子。</t>
+          <t>事件規則：每 3 回合觸發一次。預告時即高亮受影響格子。事件抽選使用加權系統，莫菲定律權重根據玩家行為動態調整。跨輪未觸發事件會保留並提前觸發回合。</t>
         </is>
       </c>
     </row>
@@ -4440,6 +4440,60 @@
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>無</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>🔀</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>莫菲定律</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>所有設施隨機打亂位置，獲得 2 張複合設施。觸發時劫持預告事件（第2輪起，權重根據重複投入/未移動設施累積）。觸發後下次事件限定池。</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>負面</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>所有設施格</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>💼</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>就業輔助</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>獲得目標 20% 收益</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>正面</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>無</t>
         </is>
@@ -4724,7 +4778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5025,6 +5079,69 @@
       <c r="C32" s="10" t="inlineStr">
         <is>
           <t>失敗重開時難度重置為 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>莫菲定律權重系統</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>觸發條件</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>第2輪起，連續同方向投入4+次（每多1次+3權重）或未移動設施6+回合（每多1回合+2權重）。機率上限60%。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>觸發方式</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>不進入預告池，事件觸發時由checkMurphyHijack()根據權重判定是否劫持替換預告事件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>觸發後效果</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>全屏特效（震動+立繪），所有設施打亂，給2張複合設施，下次事件限定池（設施補給/地震/就業輔助/蕾雅的禮物），權重重置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>收益飛行動畫系統</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>說明</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>所有非標準收益變動（合夥人onSettle、設施效果、事件）從來源位置飛向收益UI。負數紅色。profitFlyFrom/profitFlyFromCell/profitFlyFromPartner。</t>
         </is>
       </c>
     </row>

</xml_diff>